<commit_message>
Update test data with diagnosis columns and refreshed visit dates.
Adds Diagnosis 1/2 (I10/E11) to sample spreadsheets and documents the new columns in test_data/README.md.
</commit_message>
<xml_diff>
--- a/test_data/PHC-A_CURRENT.xlsx
+++ b/test_data/PHC-A_CURRENT.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="148">
   <si>
     <t>Registration Date</t>
   </si>
@@ -67,6 +67,12 @@
     <t>Blood Sugar Value</t>
   </si>
   <si>
+    <t>Diagnosis 1</t>
+  </si>
+  <si>
+    <t>Diagnosis 2</t>
+  </si>
+  <si>
     <t>29-01-2026 00:00:00</t>
   </si>
   <si>
@@ -382,67 +388,76 @@
     <t>SHC-D</t>
   </si>
   <si>
-    <t>27-12-2025 00:00:00</t>
-  </si>
-  <si>
-    <t>30-01-2026 00:00:00</t>
-  </si>
-  <si>
-    <t>03-02-2026 00:00:00</t>
-  </si>
-  <si>
-    <t>16-01-2026 00:00:00</t>
-  </si>
-  <si>
-    <t>26-01-2026 00:00:00</t>
-  </si>
-  <si>
-    <t>17-11-2025 00:00:00</t>
-  </si>
-  <si>
-    <t>25-07-2025 00:00:00</t>
-  </si>
-  <si>
-    <t>21-11-2025 00:00:00</t>
-  </si>
-  <si>
-    <t>03-11-2024 00:00:00</t>
-  </si>
-  <si>
-    <t>17-12-2024 00:00:00</t>
-  </si>
-  <si>
-    <t>01-01-2025 00:00:00</t>
-  </si>
-  <si>
-    <t>28-01-2026 00:00:00</t>
-  </si>
-  <si>
-    <t>15-12-2025 00:00:00</t>
-  </si>
-  <si>
-    <t>13-02-2026 00:00:00</t>
-  </si>
-  <si>
-    <t>17-02-2026 00:00:00</t>
-  </si>
-  <si>
-    <t>17-08-2025 00:00:00</t>
-  </si>
-  <si>
-    <t>25-09-2025 00:00:00</t>
-  </si>
-  <si>
-    <t>30-10-2025 00:00:00</t>
-  </si>
-  <si>
-    <t>17-09-2024 00:00:00</t>
-  </si>
-  <si>
-    <t>07-01-2025 00:00:00</t>
+    <t>25-05-2026 00:00:00</t>
+  </si>
+  <si>
+    <t>27-04-2026 00:00:00</t>
+  </si>
+  <si>
+    <t>30-05-2026 00:00:00</t>
+  </si>
+  <si>
+    <t>03-06-2026 00:00:00</t>
+  </si>
+  <si>
+    <t>16-05-2026 00:00:00</t>
+  </si>
+  <si>
+    <t>26-05-2026 00:00:00</t>
+  </si>
+  <si>
+    <t>17-03-2026 00:00:00</t>
+  </si>
+  <si>
+    <t>25-11-2025 00:00:00</t>
+  </si>
+  <si>
+    <t>21-03-2026 00:00:00</t>
+  </si>
+  <si>
+    <t>03-03-2025 00:00:00</t>
+  </si>
+  <si>
+    <t>17-04-2025 00:00:00</t>
+  </si>
+  <si>
+    <t>01-05-2025 00:00:00</t>
+  </si>
+  <si>
+    <t>28-05-2026 00:00:00</t>
+  </si>
+  <si>
+    <t>15-04-2026 00:00:00</t>
+  </si>
+  <si>
+    <t>29-05-2026 00:00:00</t>
+  </si>
+  <si>
+    <t>13-06-2026 00:00:00</t>
+  </si>
+  <si>
+    <t>17-06-2026 00:00:00</t>
+  </si>
+  <si>
+    <t>17-12-2025 00:00:00</t>
+  </si>
+  <si>
+    <t>28-02-2026 00:00:00</t>
+  </si>
+  <si>
+    <t>17-01-2025 00:00:00</t>
+  </si>
+  <si>
+    <t>07-05-2025 00:00:00</t>
   </si>
   <si>
     <t>FBS</t>
+  </si>
+  <si>
+    <t>I10</t>
+  </si>
+  <si>
+    <t>E11</t>
   </si>
 </sst>
 </file>
@@ -800,10 +815,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q43"/>
+  <dimension ref="A1:S43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:19">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -855,37 +870,43 @@
       <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="2" spans="1:17">
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="G2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H2">
         <v>1640879532</v>
       </c>
       <c r="J2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="M2">
         <v>116</v>
@@ -893,40 +914,40 @@
       <c r="N2">
         <v>77</v>
       </c>
-      <c r="P2" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17">
+      <c r="R2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E3">
         <v>2</v>
       </c>
       <c r="F3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G3" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H3">
         <v>9001641291</v>
       </c>
       <c r="J3" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="M3">
         <v>133</v>
@@ -934,40 +955,40 @@
       <c r="N3">
         <v>84</v>
       </c>
-      <c r="P3" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17">
+      <c r="R3" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C4" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E4">
         <v>3</v>
       </c>
       <c r="F4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G4" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H4">
         <v>4178265580</v>
       </c>
       <c r="J4" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K4" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L4" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="M4">
         <v>134</v>
@@ -975,40 +996,40 @@
       <c r="N4">
         <v>78</v>
       </c>
-      <c r="P4" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17">
+      <c r="R4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E5">
         <v>4</v>
       </c>
       <c r="F5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H5">
         <v>9004736657</v>
       </c>
       <c r="J5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="M5">
         <v>120</v>
@@ -1017,45 +1038,51 @@
         <v>80</v>
       </c>
       <c r="O5" t="s">
-        <v>37</v>
+        <v>124</v>
       </c>
       <c r="P5" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="Q5">
         <v>120</v>
       </c>
-    </row>
-    <row r="6" spans="1:17">
+      <c r="R5" t="s">
+        <v>146</v>
+      </c>
+      <c r="S5" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E6">
         <v>5</v>
       </c>
       <c r="F6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="G6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H6">
         <v>5037957603</v>
       </c>
       <c r="J6" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="M6">
         <v>120</v>
@@ -1064,45 +1091,51 @@
         <v>80</v>
       </c>
       <c r="O6" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="P6" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="Q6">
         <v>120</v>
       </c>
-    </row>
-    <row r="7" spans="1:17">
+      <c r="R6" t="s">
+        <v>146</v>
+      </c>
+      <c r="S6" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19">
       <c r="A7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B7" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E7">
         <v>6</v>
       </c>
       <c r="F7" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="G7" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H7">
         <v>7450089069</v>
       </c>
       <c r="J7" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K7" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L7" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="M7">
         <v>120</v>
@@ -1111,45 +1144,51 @@
         <v>80</v>
       </c>
       <c r="O7" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="P7" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="Q7">
         <v>120</v>
       </c>
-    </row>
-    <row r="8" spans="1:17">
+      <c r="R7" t="s">
+        <v>146</v>
+      </c>
+      <c r="S7" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E8">
         <v>7</v>
       </c>
       <c r="F8" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="G8" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H8">
         <v>5642953020</v>
       </c>
       <c r="J8" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K8" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="M8">
         <v>141</v>
@@ -1158,45 +1197,51 @@
         <v>91</v>
       </c>
       <c r="O8" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="P8" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="Q8">
         <v>130</v>
       </c>
-    </row>
-    <row r="9" spans="1:17">
+      <c r="R8" t="s">
+        <v>146</v>
+      </c>
+      <c r="S8" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B9" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C9" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E9">
         <v>8</v>
       </c>
       <c r="F9" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H9">
         <v>3767920156</v>
       </c>
       <c r="J9" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K9" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L9" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="M9">
         <v>141</v>
@@ -1205,45 +1250,51 @@
         <v>91</v>
       </c>
       <c r="O9" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="P9" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="Q9">
         <v>130</v>
       </c>
-    </row>
-    <row r="10" spans="1:17">
+      <c r="R9" t="s">
+        <v>146</v>
+      </c>
+      <c r="S9" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19">
       <c r="A10" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C10" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E10">
         <v>9</v>
       </c>
       <c r="F10" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G10" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H10">
         <v>2391944891</v>
       </c>
       <c r="J10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L10" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="M10">
         <v>141</v>
@@ -1252,42 +1303,48 @@
         <v>91</v>
       </c>
       <c r="O10" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="P10" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="Q10">
         <v>130</v>
       </c>
-    </row>
-    <row r="11" spans="1:17">
+      <c r="R10" t="s">
+        <v>146</v>
+      </c>
+      <c r="S10" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19">
       <c r="A11" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B11" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C11" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E11">
         <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="G11" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="J11" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K11" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L11" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="M11">
         <v>120</v>
@@ -1296,42 +1353,42 @@
         <v>78</v>
       </c>
       <c r="O11" t="s">
-        <v>127</v>
-      </c>
-      <c r="P11" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17">
+        <v>130</v>
+      </c>
+      <c r="R11" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19">
       <c r="A12" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B12" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C12" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E12">
         <v>11</v>
       </c>
       <c r="F12" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="G12" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H12">
         <v>3420998771</v>
       </c>
       <c r="J12" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K12" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L12" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="M12">
         <v>118</v>
@@ -1340,39 +1397,39 @@
         <v>79</v>
       </c>
       <c r="O12" t="s">
-        <v>128</v>
-      </c>
-      <c r="P12" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="13" spans="1:17">
+        <v>131</v>
+      </c>
+      <c r="R12" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C13" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E13">
         <v>12</v>
       </c>
       <c r="F13" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="J13" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K13" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L13" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="M13">
         <v>133</v>
@@ -1381,42 +1438,42 @@
         <v>75</v>
       </c>
       <c r="O13" t="s">
-        <v>129</v>
-      </c>
-      <c r="P13" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="14" spans="1:17">
+        <v>132</v>
+      </c>
+      <c r="R13" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19">
       <c r="A14" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B14" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C14" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E14">
         <v>13</v>
       </c>
       <c r="F14" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="G14" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H14">
         <v>4015464640</v>
       </c>
       <c r="J14" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K14" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L14" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="M14">
         <v>131</v>
@@ -1425,42 +1482,42 @@
         <v>80</v>
       </c>
       <c r="O14" t="s">
-        <v>130</v>
-      </c>
-      <c r="P14" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="15" spans="1:17">
+        <v>133</v>
+      </c>
+      <c r="R14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19">
       <c r="A15" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B15" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C15" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E15">
         <v>14</v>
       </c>
       <c r="F15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="G15" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H15">
         <v>2515858745</v>
       </c>
       <c r="J15" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K15" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L15" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="M15">
         <v>123</v>
@@ -1469,42 +1526,42 @@
         <v>77</v>
       </c>
       <c r="O15" t="s">
-        <v>131</v>
-      </c>
-      <c r="P15" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="16" spans="1:17">
+        <v>134</v>
+      </c>
+      <c r="R15" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19">
       <c r="A16" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B16" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C16" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E16">
         <v>15</v>
       </c>
       <c r="F16" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="G16" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H16">
         <v>2834539761</v>
       </c>
       <c r="J16" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K16" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L16" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="M16">
         <v>131</v>
@@ -1513,42 +1570,42 @@
         <v>76</v>
       </c>
       <c r="O16" t="s">
-        <v>132</v>
-      </c>
-      <c r="P16" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17">
+        <v>135</v>
+      </c>
+      <c r="R16" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19">
       <c r="A17" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B17" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C17" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E17">
         <v>16</v>
       </c>
       <c r="F17" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="G17" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H17">
         <v>2519605117</v>
       </c>
       <c r="J17" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K17" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L17" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="M17">
         <v>134</v>
@@ -1556,37 +1613,37 @@
       <c r="N17">
         <v>78</v>
       </c>
-      <c r="P17" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17">
+      <c r="R17" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19">
       <c r="A18" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B18" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C18" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E18">
         <v>17</v>
       </c>
       <c r="F18" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G18" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="J18" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K18" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L18" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="M18">
         <v>132</v>
@@ -1594,37 +1651,37 @@
       <c r="N18">
         <v>84</v>
       </c>
-      <c r="P18" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="19" spans="1:17">
+      <c r="R18" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19">
       <c r="A19" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B19" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C19" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E19">
         <v>18</v>
       </c>
       <c r="F19" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="G19" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="J19" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K19" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L19" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="M19">
         <v>118</v>
@@ -1632,37 +1689,37 @@
       <c r="N19">
         <v>78</v>
       </c>
-      <c r="P19" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17">
+      <c r="R19" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19">
       <c r="A20" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B20" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C20" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E20">
         <v>19</v>
       </c>
       <c r="F20" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G20" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="J20" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K20" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L20" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="M20">
         <v>117</v>
@@ -1670,37 +1727,37 @@
       <c r="N20">
         <v>85</v>
       </c>
-      <c r="P20" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17">
+      <c r="R20" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19">
       <c r="A21" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B21" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C21" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E21">
         <v>20</v>
       </c>
       <c r="F21" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="G21" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="J21" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K21" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L21" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="M21">
         <v>134</v>
@@ -1708,40 +1765,40 @@
       <c r="N21">
         <v>76</v>
       </c>
-      <c r="P21" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="22" spans="1:17">
+      <c r="R21" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19">
       <c r="A22" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B22" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C22" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E22">
         <v>21</v>
       </c>
       <c r="F22" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="G22" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H22">
         <v>4291035954</v>
       </c>
       <c r="J22" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K22" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L22" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="M22">
         <v>135</v>
@@ -1749,40 +1806,40 @@
       <c r="N22">
         <v>80</v>
       </c>
-      <c r="P22" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="23" spans="1:17">
+      <c r="R22" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19">
       <c r="A23" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B23" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C23" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E23">
         <v>22</v>
       </c>
       <c r="F23" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="G23" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H23">
         <v>1640879532</v>
       </c>
       <c r="J23" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K23" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L23" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="M23">
         <v>123</v>
@@ -1790,40 +1847,40 @@
       <c r="N23">
         <v>85</v>
       </c>
-      <c r="P23" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="24" spans="1:17">
+      <c r="R23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19">
       <c r="A24" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C24" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E24">
         <v>23</v>
       </c>
       <c r="F24" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G24" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H24">
         <v>9001641291</v>
       </c>
       <c r="J24" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K24" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L24" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="M24">
         <v>134</v>
@@ -1831,40 +1888,40 @@
       <c r="N24">
         <v>77</v>
       </c>
-      <c r="P24" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="25" spans="1:17">
+      <c r="R24" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19">
       <c r="A25" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B25" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C25" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E25">
         <v>24</v>
       </c>
       <c r="F25" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G25" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H25">
         <v>4178265580</v>
       </c>
       <c r="J25" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K25" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L25" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="M25">
         <v>121</v>
@@ -1872,40 +1929,40 @@
       <c r="N25">
         <v>78</v>
       </c>
-      <c r="P25" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="26" spans="1:17">
+      <c r="R25" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19">
       <c r="A26" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B26" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C26" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E26">
         <v>29</v>
       </c>
       <c r="F26" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G26" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H26">
         <v>3767920156</v>
       </c>
       <c r="J26" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K26" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L26" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="M26">
         <v>120</v>
@@ -1914,45 +1971,51 @@
         <v>80</v>
       </c>
       <c r="O26" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="P26" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="Q26">
         <v>120</v>
       </c>
-    </row>
-    <row r="27" spans="1:17">
+      <c r="R26" t="s">
+        <v>146</v>
+      </c>
+      <c r="S26" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19">
       <c r="A27" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B27" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E27">
         <v>25</v>
       </c>
       <c r="F27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G27" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H27">
         <v>9004736657</v>
       </c>
       <c r="J27" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K27" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="M27">
         <v>120</v>
@@ -1961,45 +2024,51 @@
         <v>80</v>
       </c>
       <c r="O27" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="P27" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="Q27">
         <v>120</v>
       </c>
-    </row>
-    <row r="28" spans="1:17">
+      <c r="R27" t="s">
+        <v>146</v>
+      </c>
+      <c r="S27" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19">
       <c r="A28" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B28" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C28" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E28">
         <v>26</v>
       </c>
       <c r="F28" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="G28" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H28">
         <v>5037957603</v>
       </c>
       <c r="J28" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K28" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L28" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="M28">
         <v>120</v>
@@ -2008,45 +2077,51 @@
         <v>80</v>
       </c>
       <c r="O28" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="P28" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="Q28">
         <v>120</v>
       </c>
-    </row>
-    <row r="29" spans="1:17">
+      <c r="R28" t="s">
+        <v>146</v>
+      </c>
+      <c r="S28" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="29" spans="1:19">
       <c r="A29" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B29" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C29" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E29">
         <v>27</v>
       </c>
       <c r="F29" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="G29" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H29">
         <v>7450089069</v>
       </c>
       <c r="J29" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K29" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L29" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="M29">
         <v>141</v>
@@ -2055,45 +2130,51 @@
         <v>91</v>
       </c>
       <c r="O29" t="s">
-        <v>17</v>
+        <v>138</v>
       </c>
       <c r="P29" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="Q29">
         <v>130</v>
       </c>
-    </row>
-    <row r="30" spans="1:17">
+      <c r="R29" t="s">
+        <v>146</v>
+      </c>
+      <c r="S29" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="30" spans="1:19">
       <c r="A30" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B30" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C30" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E30">
         <v>28</v>
       </c>
       <c r="F30" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="G30" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H30">
         <v>5642953020</v>
       </c>
       <c r="J30" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K30" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L30" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="M30">
         <v>141</v>
@@ -2102,45 +2183,51 @@
         <v>91</v>
       </c>
       <c r="O30" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="P30" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="Q30">
         <v>130</v>
       </c>
-    </row>
-    <row r="31" spans="1:17">
+      <c r="R30" t="s">
+        <v>146</v>
+      </c>
+      <c r="S30" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="31" spans="1:19">
       <c r="A31" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B31" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C31" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E31">
         <v>30</v>
       </c>
       <c r="F31" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G31" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H31">
         <v>2391944891</v>
       </c>
       <c r="J31" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K31" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L31" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="M31">
         <v>141</v>
@@ -2149,42 +2236,48 @@
         <v>91</v>
       </c>
       <c r="O31" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="P31" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="Q31">
         <v>130</v>
       </c>
-    </row>
-    <row r="32" spans="1:17">
+      <c r="R31" t="s">
+        <v>146</v>
+      </c>
+      <c r="S31" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="32" spans="1:19">
       <c r="A32" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B32" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C32" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E32">
         <v>31</v>
       </c>
       <c r="F32" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="G32" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="J32" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K32" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L32" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="M32">
         <v>132</v>
@@ -2193,42 +2286,42 @@
         <v>76</v>
       </c>
       <c r="O32" t="s">
-        <v>137</v>
-      </c>
-      <c r="P32" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="33" spans="1:16">
+        <v>141</v>
+      </c>
+      <c r="R32" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="33" spans="1:18">
       <c r="A33" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B33" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C33" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E33">
         <v>32</v>
       </c>
       <c r="F33" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="G33" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H33">
         <v>3420998771</v>
       </c>
       <c r="J33" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K33" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L33" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="M33">
         <v>133</v>
@@ -2237,39 +2330,39 @@
         <v>82</v>
       </c>
       <c r="O33" t="s">
-        <v>138</v>
-      </c>
-      <c r="P33" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="34" spans="1:16">
+        <v>39</v>
+      </c>
+      <c r="R33" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="34" spans="1:18">
       <c r="A34" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B34" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C34" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E34">
         <v>33</v>
       </c>
       <c r="F34" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G34" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="J34" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K34" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L34" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="M34">
         <v>119</v>
@@ -2278,42 +2371,42 @@
         <v>77</v>
       </c>
       <c r="O34" t="s">
-        <v>139</v>
-      </c>
-      <c r="P34" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="35" spans="1:16">
+      <c r="R34" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18">
       <c r="A35" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B35" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C35" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E35">
         <v>34</v>
       </c>
       <c r="F35" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="G35" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H35">
         <v>4015464640</v>
       </c>
       <c r="J35" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K35" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L35" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="M35">
         <v>130</v>
@@ -2322,42 +2415,42 @@
         <v>77</v>
       </c>
       <c r="O35" t="s">
-        <v>130</v>
-      </c>
-      <c r="P35" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="36" spans="1:16">
+        <v>133</v>
+      </c>
+      <c r="R35" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18">
       <c r="A36" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B36" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C36" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E36">
         <v>35</v>
       </c>
       <c r="F36" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="G36" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H36">
         <v>2515858745</v>
       </c>
       <c r="J36" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K36" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L36" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="M36">
         <v>118</v>
@@ -2366,42 +2459,42 @@
         <v>78</v>
       </c>
       <c r="O36" t="s">
-        <v>140</v>
-      </c>
-      <c r="P36" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="37" spans="1:16">
+        <v>143</v>
+      </c>
+      <c r="R36" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18">
       <c r="A37" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B37" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C37" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E37">
         <v>36</v>
       </c>
       <c r="F37" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="G37" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H37">
         <v>2834539761</v>
       </c>
       <c r="J37" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K37" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L37" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="M37">
         <v>131</v>
@@ -2410,42 +2503,42 @@
         <v>76</v>
       </c>
       <c r="O37" t="s">
-        <v>141</v>
-      </c>
-      <c r="P37" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="38" spans="1:16">
+        <v>144</v>
+      </c>
+      <c r="R37" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="38" spans="1:18">
       <c r="A38" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B38" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C38" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E38">
         <v>37</v>
       </c>
       <c r="F38" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="G38" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H38">
         <v>2519605117</v>
       </c>
       <c r="J38" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K38" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L38" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="M38">
         <v>131</v>
@@ -2453,37 +2546,37 @@
       <c r="N38">
         <v>82</v>
       </c>
-      <c r="P38" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="39" spans="1:16">
+      <c r="R38" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="39" spans="1:18">
       <c r="A39" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B39" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C39" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E39">
         <v>38</v>
       </c>
       <c r="F39" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G39" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="J39" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K39" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L39" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="M39">
         <v>120</v>
@@ -2491,37 +2584,37 @@
       <c r="N39">
         <v>84</v>
       </c>
-      <c r="P39" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="40" spans="1:16">
+      <c r="R39" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="40" spans="1:18">
       <c r="A40" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B40" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C40" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E40">
         <v>39</v>
       </c>
       <c r="F40" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="G40" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="J40" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K40" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L40" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="M40">
         <v>117</v>
@@ -2529,37 +2622,37 @@
       <c r="N40">
         <v>83</v>
       </c>
-      <c r="P40" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="41" spans="1:16">
+      <c r="R40" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="41" spans="1:18">
       <c r="A41" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B41" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C41" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E41">
         <v>40</v>
       </c>
       <c r="F41" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G41" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="J41" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K41" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L41" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="M41">
         <v>115</v>
@@ -2567,37 +2660,37 @@
       <c r="N41">
         <v>84</v>
       </c>
-      <c r="P41" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="42" spans="1:16">
+      <c r="R41" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="42" spans="1:18">
       <c r="A42" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B42" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C42" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E42">
         <v>41</v>
       </c>
       <c r="F42" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="G42" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="J42" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K42" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L42" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="M42">
         <v>116</v>
@@ -2605,40 +2698,40 @@
       <c r="N42">
         <v>78</v>
       </c>
-      <c r="P42" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="43" spans="1:16">
+      <c r="R42" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="43" spans="1:18">
       <c r="A43" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B43" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C43" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E43">
         <v>42</v>
       </c>
       <c r="F43" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="G43" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H43">
         <v>4291035954</v>
       </c>
       <c r="J43" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K43" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L43" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="M43">
         <v>123</v>
@@ -2646,8 +2739,8 @@
       <c r="N43">
         <v>80</v>
       </c>
-      <c r="P43" t="s">
-        <v>142</v>
+      <c r="R43" t="s">
+        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>